<commit_message>
Added propagation of calc chain ofr template v2, code discrepancies now during loading, error table replaced with arithmetic mean
</commit_message>
<xml_diff>
--- a/inst/extdata/mocaredd-templatev2-4pools.xlsx
+++ b/inst/extdata/mocaredd-templatev2-4pools.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gaelsola/code/mocaredd.dev2/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE3B16C-8B9F-8445-B195-D91BB469E0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEE6420-0D74-3A45-84AD-F0E0AA8A3904}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33220" yWindow="-6940" windowWidth="28200" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23000" yWindow="600" windowWidth="28200" windowHeight="18460" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="11" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="79">
   <si>
     <t>trans_no</t>
   </si>
@@ -485,6 +485,9 @@
       <t>(*): "Degraded".
 (*) In this paragraph xx/yy means TAB_NAME/COLUMN_NAME.</t>
     </r>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1110,7 @@
         <v>2020</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>43</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.15">
@@ -2584,20 +2587,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="35.33203125" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="19" t="s">
         <v>10</v>
       </c>
@@ -2605,31 +2608,34 @@
         <v>44</v>
       </c>
       <c r="C1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="19" t="s">
-        <v>51</v>
-      </c>
       <c r="E1" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="G1" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="H1" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="I1" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="J1" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="19" t="s">
+      <c r="K1" s="19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2637,25 +2643,28 @@
         <v>23</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="4">
+      <c r="E2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="4">
         <v>28.72</v>
       </c>
-      <c r="F2" s="4">
+      <c r="G2" s="4">
         <v>5.62</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H2" s="4"/>
+      <c r="H2" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -2663,25 +2672,28 @@
         <v>23</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="E3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="4">
         <v>85.34</v>
       </c>
-      <c r="F3" s="4">
+      <c r="G3" s="4">
         <v>45.6</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H3" s="4"/>
+      <c r="H3" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -2689,25 +2701,28 @@
         <v>23</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="E4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="4">
         <v>212.99</v>
       </c>
-      <c r="F4" s="4">
+      <c r="G4" s="4">
         <v>43.58</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -2715,25 +2730,28 @@
         <v>23</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="4">
+      <c r="E5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="4">
         <v>105.48</v>
       </c>
-      <c r="F5" s="4">
+      <c r="G5" s="4">
         <v>37.049999999999997</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
-    </row>
-    <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K5" s="4"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -2741,25 +2759,28 @@
         <v>23</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="4">
+      <c r="E6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="4">
         <v>79.709999999999994</v>
       </c>
-      <c r="F6" s="4">
+      <c r="G6" s="4">
         <v>11.55</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H6" s="4"/>
+      <c r="H6" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
-    </row>
-    <row r="7" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K6" s="4"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -2767,25 +2788,28 @@
         <v>23</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E7" s="4">
+      <c r="E7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="4">
         <v>78.33</v>
       </c>
-      <c r="F7" s="4">
+      <c r="G7" s="4">
         <v>14.56</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H7" s="4"/>
+      <c r="H7" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
-    </row>
-    <row r="8" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K7" s="4"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2793,25 +2817,28 @@
         <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="5">
+      <c r="E8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="5">
         <v>10.89</v>
       </c>
-      <c r="F8" s="5">
+      <c r="G8" s="5">
         <v>1.94</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K8" s="5"/>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2819,25 +2846,28 @@
         <v>23</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" s="5">
+      <c r="E9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="5">
         <v>11.03</v>
       </c>
-      <c r="F9" s="5">
+      <c r="G9" s="5">
         <v>5.24</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H9" s="5"/>
+      <c r="H9" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -2845,25 +2875,28 @@
         <v>23</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="5">
+      <c r="E10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="5">
         <v>28.12</v>
       </c>
-      <c r="F10" s="5">
+      <c r="G10" s="5">
         <v>5.84</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" s="5"/>
+      <c r="H10" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2871,25 +2904,28 @@
         <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="5">
+      <c r="E11" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="5">
         <v>27.14</v>
       </c>
-      <c r="F11" s="5">
+      <c r="G11" s="5">
         <v>3.8</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H11" s="5"/>
+      <c r="H11" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2897,25 +2933,28 @@
         <v>23</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E12" s="5">
+      <c r="E12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="5">
         <v>19.940000000000001</v>
       </c>
-      <c r="F12" s="5">
+      <c r="G12" s="5">
         <v>2.2400000000000002</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" s="5"/>
+      <c r="H12" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K12" s="5"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -2923,25 +2962,28 @@
         <v>23</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E13" s="5">
+      <c r="E13" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="5">
         <v>25.29</v>
       </c>
-      <c r="F13" s="5">
+      <c r="G13" s="5">
         <v>2.4700000000000002</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K13" s="5"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -2949,25 +2991,28 @@
         <v>23</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="4">
+      <c r="E14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="4">
         <v>21.53</v>
       </c>
-      <c r="F14" s="4">
+      <c r="G14" s="4">
         <v>4.45</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H14" s="4"/>
+      <c r="H14" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K14" s="4"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -2975,25 +3020,28 @@
         <v>23</v>
       </c>
       <c r="C15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="4">
+      <c r="E15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="4">
         <v>30.42</v>
       </c>
-      <c r="F15" s="4">
+      <c r="G15" s="4">
         <v>25.56</v>
       </c>
-      <c r="G15" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H15" s="4"/>
+      <c r="H15" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-    </row>
-    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K15" s="4"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -3001,25 +3049,28 @@
         <v>23</v>
       </c>
       <c r="C16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="4">
+      <c r="E16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="4">
         <v>19.2</v>
       </c>
-      <c r="F16" s="4">
+      <c r="G16" s="4">
         <v>6.75</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H16" s="4"/>
+      <c r="H16" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-    </row>
-    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -3027,25 +3078,28 @@
         <v>23</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E17" s="4">
+      <c r="E17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F17" s="4">
         <v>69.12</v>
       </c>
-      <c r="F17" s="4">
+      <c r="G17" s="4">
         <v>23.29</v>
       </c>
-      <c r="G17" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H17" s="4"/>
+      <c r="H17" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
-    </row>
-    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -3053,25 +3107,28 @@
         <v>23</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" s="4">
+      <c r="E18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="4">
         <v>40.549999999999997</v>
       </c>
-      <c r="F18" s="4">
+      <c r="G18" s="4">
         <v>7.76</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H18" s="4"/>
+      <c r="H18" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
-    </row>
-    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -3079,25 +3136,28 @@
         <v>23</v>
       </c>
       <c r="C19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E19" s="4">
+      <c r="E19" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="4">
         <v>44.03</v>
       </c>
-      <c r="F19" s="4">
+      <c r="G19" s="4">
         <v>14.81</v>
       </c>
-      <c r="G19" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H19" s="4"/>
+      <c r="H19" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I19" s="4"/>
       <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -3105,25 +3165,28 @@
         <v>23</v>
       </c>
       <c r="C20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="5">
+      <c r="E20" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="5">
         <v>2.73</v>
       </c>
-      <c r="F20" s="5">
+      <c r="G20" s="5">
         <v>0.41</v>
       </c>
-      <c r="G20" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H20" s="5"/>
+      <c r="H20" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -3131,25 +3194,28 @@
         <v>23</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="5">
+      <c r="E21" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="5">
         <v>3.13</v>
       </c>
-      <c r="F21" s="5">
+      <c r="G21" s="5">
         <v>0.42</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -3157,25 +3223,28 @@
         <v>23</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="5">
+      <c r="E22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="5">
         <v>3.48</v>
       </c>
-      <c r="F22" s="5">
+      <c r="G22" s="5">
         <v>1.07</v>
       </c>
-      <c r="G22" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H22" s="5"/>
+      <c r="H22" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -3183,25 +3252,28 @@
         <v>23</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E23" s="5">
+      <c r="E23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="5">
         <v>3.06</v>
       </c>
-      <c r="F23" s="5">
+      <c r="G23" s="5">
         <v>0.47</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H23" s="5"/>
+      <c r="H23" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -3209,25 +3281,28 @@
         <v>23</v>
       </c>
       <c r="C24" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="5">
+      <c r="E24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="5">
         <v>2.52</v>
       </c>
-      <c r="F24" s="5">
+      <c r="G24" s="5">
         <v>0.36</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H24" s="5"/>
+      <c r="H24" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -3235,25 +3310,28 @@
         <v>23</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" s="5">
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="5">
         <v>1.45</v>
       </c>
-      <c r="F25" s="5">
+      <c r="G25" s="5">
         <v>0.26</v>
       </c>
-      <c r="G25" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="H25" s="5"/>
+      <c r="H25" s="5" t="s">
+        <v>63</v>
+      </c>
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -3261,25 +3339,28 @@
         <v>23</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="4">
+        <v>23</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="4">
         <v>15.02</v>
       </c>
-      <c r="F26" s="4">
+      <c r="G26" s="4">
         <v>16.96</v>
       </c>
-      <c r="G26" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H26" s="4"/>
+      <c r="H26" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
-    </row>
-    <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -3287,25 +3368,28 @@
         <v>23</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E27" s="4">
+        <v>23</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="4">
         <v>15.95</v>
       </c>
-      <c r="F27" s="4">
+      <c r="G27" s="4">
         <v>15.34</v>
       </c>
-      <c r="G27" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H27" s="4"/>
+      <c r="H27" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
-    </row>
-    <row r="28" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K27" s="4"/>
+    </row>
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -3313,25 +3397,28 @@
         <v>23</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="E28" s="4">
+        <v>23</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="4">
         <v>17.809999999999999</v>
       </c>
-      <c r="F28" s="4">
+      <c r="G28" s="4">
         <v>8.26</v>
       </c>
-      <c r="G28" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H28" s="4"/>
+      <c r="H28" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K28" s="4"/>
+    </row>
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -3339,25 +3426,28 @@
         <v>23</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E29" s="4">
+        <v>23</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="4">
         <v>14.52</v>
       </c>
-      <c r="F29" s="4">
+      <c r="G29" s="4">
         <v>6.78</v>
       </c>
-      <c r="G29" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H29" s="4"/>
+      <c r="H29" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
-    </row>
-    <row r="30" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K29" s="4"/>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -3365,25 +3455,28 @@
         <v>23</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E30" s="4">
+        <v>23</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="4">
         <v>18.5</v>
       </c>
-      <c r="F30" s="4">
+      <c r="G30" s="4">
         <v>7.28</v>
       </c>
-      <c r="G30" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H30" s="4"/>
+      <c r="H30" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K30" s="4"/>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -3391,25 +3484,28 @@
         <v>23</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E31" s="4">
+        <v>23</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="4">
         <v>8.3000000000000007</v>
       </c>
-      <c r="F31" s="4">
+      <c r="G31" s="4">
         <v>8.75</v>
       </c>
-      <c r="G31" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="H31" s="4"/>
+      <c r="H31" s="4" t="s">
+        <v>63</v>
+      </c>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
-    </row>
-    <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K31" s="4"/>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -3417,31 +3513,34 @@
         <v>23</v>
       </c>
       <c r="C32" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E32" s="5">
+      <c r="E32" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F32" s="5">
         <v>0.55000000000000004</v>
       </c>
-      <c r="F32" s="5">
+      <c r="G32" s="5">
         <v>0.08</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="H32" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H32" s="5">
-        <f>ROUND((E32*(1-E32)/(F32*F32)-1)*E32,2)</f>
+      <c r="I32" s="5">
+        <f>ROUND((F32*(1-F32)/(G32*G32)-1)*F32,2)</f>
         <v>20.72</v>
       </c>
-      <c r="I32" s="5">
-        <f>ROUND((E32*(1-E32)/(F32*F32)-1)*(1-E32),2)</f>
+      <c r="J32" s="5">
+        <f>ROUND((F32*(1-F32)/(G32*G32)-1)*(1-F32),2)</f>
         <v>16.95</v>
       </c>
-      <c r="J32" s="5"/>
-    </row>
-    <row r="33" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -3449,31 +3548,34 @@
         <v>23</v>
       </c>
       <c r="C33" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E33" s="5">
+      <c r="E33" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F33" s="5">
         <v>0.74</v>
       </c>
-      <c r="F33" s="5">
+      <c r="G33" s="5">
         <v>0.02</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="H33" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H33" s="5">
-        <f t="shared" ref="H33:H37" si="0">ROUND((E33*(1-E33)/(F33*F33)-1)*E33,2)</f>
+      <c r="I33" s="5">
+        <f t="shared" ref="I33:I37" si="0">ROUND((F33*(1-F33)/(G33*G33)-1)*F33,2)</f>
         <v>355.2</v>
       </c>
-      <c r="I33" s="5">
-        <f t="shared" ref="I33:I37" si="1">ROUND((E33*(1-E33)/(F33*F33)-1)*(1-E33),2)</f>
+      <c r="J33" s="5">
+        <f t="shared" ref="J33:J37" si="1">ROUND((F33*(1-F33)/(G33*G33)-1)*(1-F33),2)</f>
         <v>124.8</v>
       </c>
-      <c r="J33" s="5"/>
-    </row>
-    <row r="34" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -3481,31 +3583,34 @@
         <v>23</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E34" s="5">
+      <c r="E34" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F34" s="5">
         <v>0.74</v>
       </c>
-      <c r="F34" s="5">
+      <c r="G34" s="5">
         <v>0.03</v>
       </c>
-      <c r="G34" s="5" t="s">
+      <c r="H34" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H34" s="5">
+      <c r="I34" s="5">
         <f t="shared" si="0"/>
         <v>157.46</v>
       </c>
-      <c r="I34" s="5">
+      <c r="J34" s="5">
         <f t="shared" si="1"/>
         <v>55.32</v>
       </c>
-      <c r="J34" s="5"/>
-    </row>
-    <row r="35" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -3513,31 +3618,34 @@
         <v>23</v>
       </c>
       <c r="C35" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E35" s="5">
+      <c r="E35" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F35" s="5">
         <v>0.74</v>
       </c>
-      <c r="F35" s="5">
+      <c r="G35" s="5">
         <v>0.03</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="H35" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H35" s="5">
+      <c r="I35" s="5">
         <f t="shared" si="0"/>
         <v>157.46</v>
       </c>
-      <c r="I35" s="5">
+      <c r="J35" s="5">
         <f t="shared" si="1"/>
         <v>55.32</v>
       </c>
-      <c r="J35" s="5"/>
-    </row>
-    <row r="36" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -3545,31 +3653,34 @@
         <v>23</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="5">
+      <c r="E36" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F36" s="5">
         <v>0.74</v>
       </c>
-      <c r="F36" s="5">
+      <c r="G36" s="5">
         <v>0.02</v>
       </c>
-      <c r="G36" s="5" t="s">
+      <c r="H36" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H36" s="5">
+      <c r="I36" s="5">
         <f t="shared" si="0"/>
         <v>355.2</v>
       </c>
-      <c r="I36" s="5">
+      <c r="J36" s="5">
         <f t="shared" si="1"/>
         <v>124.8</v>
       </c>
-      <c r="J36" s="5"/>
-    </row>
-    <row r="37" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -3577,33 +3688,36 @@
         <v>23</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E37" s="5">
+      <c r="E37" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="5">
         <v>0.74</v>
       </c>
-      <c r="F37" s="5">
+      <c r="G37" s="5">
         <v>0.03</v>
       </c>
-      <c r="G37" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="H37" s="5">
+      <c r="I37" s="5">
         <f t="shared" si="0"/>
         <v>157.46</v>
       </c>
-      <c r="I37" s="5">
+      <c r="J37" s="5">
         <f t="shared" si="1"/>
         <v>55.32</v>
       </c>
-      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C31" xr:uid="{3D7EF7D9-A43C-A04A-950F-6332D8AE5CD1}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D31" xr:uid="{3D7EF7D9-A43C-A04A-950F-6332D8AE5CD1}">
       <formula1>"AGB,BGB,DW,LI,SOC,ALL"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>